<commit_message>
Fix Aubrey/Reid/Napa heroes and ASCII inch marks in imports
- Aubrey dining mains: full-set lifestyle shots
- Reid dining mains: full-set lifestyle; black server RED500KSV fixed
  (also mirrored to SS-RED600KSV)
- Napa SS-NP500-5PC: dining set instead of bar/stool console
- Replace Unicode inches/bullets/dashes with ASCII so Volusion
  stops showing "?" in names and descriptions

Co-authored-by: emcc10 <emcc10@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/imports/steve-silver-volusion/McCabe_SteveSilver_Import.xlsx
+++ b/docs/imports/steve-silver-volusion/McCabe_SteveSilver_Import.xlsx
@@ -466,7 +466,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Artemis 5-Piece 70″ Rect Gray Marble Table, Black Finish w/4 Black Vegan Leather Chairs</t>
+          <t>Artemis 5-Piece 70" Rect Gray Marble Table, Black Finish w/4 Black Vegan Leather Chairs</t>
         </is>
       </c>
       <c r="C2" t="inlineStr"/>
@@ -483,23 +483,23 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Meet the Artemis 70-inch marble top table—where modern design feels both elegant and inviting. Its architectural base makes a bold statement, while the sophisticated black finish keeps the look relaxed and livable. The sleek gray marble top adds a refined touch. Paired with soft black vegan leather chairs, each with a perfectly pitched seat for comfort, it’s made for gathering. Built with solid wood legs and screwed corner joints, this set offers lasting durability with effortless style.</t>
+          <t>Meet the Artemis 70-inch marble top table-where modern design feels both elegant and inviting. Its architectural base makes a bold statement, while the sophisticated black finish keeps the look relaxed and livable. The sleek gray marble top adds a refined touch. Paired with soft black vegan leather chairs, each with a perfectly pitched seat for comfort, it's made for gathering. Built with solid wood legs and screwed corner joints, this set offers lasting durability with effortless style.</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>• Expertly crafted of gray marble veneers, ash veneers, solid Asian hardwoods and engineered woods, 100% polyester and foam
-• 5-piece set includes the Artemis 70″ Gray Marble Dining Table, Black Finish and 4 Artemis Black Vegan Leather Side Chairs. Each item also sold separately.
-• Kiln-dried wood helps prevent warping, splitting and cracking
-• The chairs are solidly constructed using mortise-and-tenon joinery, corner blocks, sturdy solid wood legs, and screwed joints, this piece delivers exceptional stability, longevity, and superior furniture integrity with a 250 lb. weight capacity ensures durability and reliable support for the chair.
-• The chair legs are hand-stained in a natural multi-step black finish to highlight the natural grain and knots of the wood
-• Plastic glides help prevent scratches or mars to floors
-• The chair’s sleek black vegan leather, made from 100% polyester, offers the look and feel of real leather with easy-care convenience.
-• Available in green velvet, brown velvet, beige chenille, gray chenille, gray vegan leather and black vegan leather; in counter and dining height sizes
-• Chairs are packed 2 per carton
-• Each marble top is crafted by nature with unique characteristics that vary slightly so no two pieces will be exactly alike
-• 70″ long table seats six comfortably
-• The wood is hand-stained in a natural multi-step black finish to highlight the natural grain and knots of the wood</t>
+          <t>* Expertly crafted of gray marble veneers, ash veneers, solid Asian hardwoods and engineered woods, 100% polyester and foam
+* 5-piece set includes the Artemis 70" Gray Marble Dining Table, Black Finish and 4 Artemis Black Vegan Leather Side Chairs. Each item also sold separately.
+* Kiln-dried wood helps prevent warping, splitting and cracking
+* The chairs are solidly constructed using mortise-and-tenon joinery, corner blocks, sturdy solid wood legs, and screwed joints, this piece delivers exceptional stability, longevity, and superior furniture integrity with a 250 lb. weight capacity ensures durability and reliable support for the chair.
+* The chair legs are hand-stained in a natural multi-step black finish to highlight the natural grain and knots of the wood
+* Plastic glides help prevent scratches or mars to floors
+* The chair's sleek black vegan leather, made from 100% polyester, offers the look and feel of real leather with easy-care convenience.
+* Available in green velvet, brown velvet, beige chenille, gray chenille, gray vegan leather and black vegan leather; in counter and dining height sizes
+* Chairs are packed 2 per carton
+* Each marble top is crafted by nature with unique characteristics that vary slightly so no two pieces will be exactly alike
+* 70" long table seats six comfortably
+* The wood is hand-stained in a natural multi-step black finish to highlight the natural grain and knots of the wood</t>
         </is>
       </c>
     </row>
@@ -511,7 +511,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Artemis 5-Piece 70″ Rect Gray Marble Table, Black Finish w/4 White Vegan Leather Chairs</t>
+          <t>Artemis 5-Piece 70" Rect Gray Marble Table, Black Finish w/4 White Vegan Leather Chairs</t>
         </is>
       </c>
       <c r="C3" t="inlineStr"/>
@@ -528,23 +528,23 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Meet the Artemis 70-inch marble top table—where modern design feels both elegant and inviting. Its architectural base makes a bold statement, while the sophisticated black finish keeps the look relaxed and livable. The sleek gray marble top adds a refined touch. Paired with soft white vegan leather chairs, each with a perfectly pitched seat for comfort, it’s made for gathering. Built with solid wood legs and screwed corner joints, this set offers lasting durability with effortless style.</t>
+          <t>Meet the Artemis 70-inch marble top table-where modern design feels both elegant and inviting. Its architectural base makes a bold statement, while the sophisticated black finish keeps the look relaxed and livable. The sleek gray marble top adds a refined touch. Paired with soft white vegan leather chairs, each with a perfectly pitched seat for comfort, it's made for gathering. Built with solid wood legs and screwed corner joints, this set offers lasting durability with effortless style.</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>• Expertly crafted of gray marble veneers, ash veneers, solid Asian hardwoods and engineered woods, 100% polyester and foam
-• 5-piece set includes the Artemis 70″ Gray Marble Dining Table, Black Finish and 4 Artemis White Vegan Leather Side Chairs. Each item also sold separately.
-• Kiln-dried wood helps prevent warping, splitting and cracking
-• The chairs are solidly constructed using mortise-and-tenon joinery, corner blocks, sturdy solid wood legs, and screwed joints, this piece delivers exceptional stability, longevity, and superior furniture integrity with a 250 lb. weight capacity ensures durability and reliable support for the chair.
-• The chair legs are hand-stained in a natural multi-step black finish to highlight the natural grain and knots of the wood
-• Plastic glides help prevent scratches or mars to floors
-• The chair’s sleek white vegan leather, made from 100% polyester, offers the look and feel of real leather with easy-care convenience.
-• Available in green velvet, brown velvet, beige chenille, gray chenille, white vegan leather and black vegan leather; in counter and dining height sizes
-• Chairs are packed 2 per carton
-• Each marble top is crafted by nature with unique characteristics that vary slightly so no two pieces will be exactly alike
-• 70″ long table seats six comfortably
-• The wood is hand-stained in a natural multi-step black finish to highlight the natural grain and knots of the wood</t>
+          <t>* Expertly crafted of gray marble veneers, ash veneers, solid Asian hardwoods and engineered woods, 100% polyester and foam
+* 5-piece set includes the Artemis 70" Gray Marble Dining Table, Black Finish and 4 Artemis White Vegan Leather Side Chairs. Each item also sold separately.
+* Kiln-dried wood helps prevent warping, splitting and cracking
+* The chairs are solidly constructed using mortise-and-tenon joinery, corner blocks, sturdy solid wood legs, and screwed joints, this piece delivers exceptional stability, longevity, and superior furniture integrity with a 250 lb. weight capacity ensures durability and reliable support for the chair.
+* The chair legs are hand-stained in a natural multi-step black finish to highlight the natural grain and knots of the wood
+* Plastic glides help prevent scratches or mars to floors
+* The chair's sleek white vegan leather, made from 100% polyester, offers the look and feel of real leather with easy-care convenience.
+* Available in green velvet, brown velvet, beige chenille, gray chenille, white vegan leather and black vegan leather; in counter and dining height sizes
+* Chairs are packed 2 per carton
+* Each marble top is crafted by nature with unique characteristics that vary slightly so no two pieces will be exactly alike
+* 70" long table seats six comfortably
+* The wood is hand-stained in a natural multi-step black finish to highlight the natural grain and knots of the wood</t>
         </is>
       </c>
     </row>
@@ -556,7 +556,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Artemis 5 Piece 70″ Rect White Marble Table, Black Finish w/4 Black Vegan Leather Chairs</t>
+          <t>Artemis 5 Piece 70" Rect White Marble Table, Black Finish w/4 Black Vegan Leather Chairs</t>
         </is>
       </c>
       <c r="C4" t="inlineStr"/>
@@ -573,23 +573,23 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Meet the Artemis 70-inch marble top table—where modern design feels both elegant and inviting. Its architectural base makes a bold statement, while the sophisticated black finish keeps the look relaxed and livable. The sleek white marble top adds a refined touch. Paired with soft black vegan leather chairs, each with a perfectly pitched seat for comfort, it’s made for gathering. Built with solid wood legs and screwed corner joints, this set offers lasting durability with effortless style.</t>
+          <t>Meet the Artemis 70-inch marble top table-where modern design feels both elegant and inviting. Its architectural base makes a bold statement, while the sophisticated black finish keeps the look relaxed and livable. The sleek white marble top adds a refined touch. Paired with soft black vegan leather chairs, each with a perfectly pitched seat for comfort, it's made for gathering. Built with solid wood legs and screwed corner joints, this set offers lasting durability with effortless style.</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>• Expertly crafted of white marble veneers, ash veneers, solid Asian hardwoods and engineered woods, 100% polyester and foam
-• 5-piece set includes the Artemis 70″ White Marble Dining Table, Black Finish and 4 Artemis Black Vegan Leather Side Chairs. Each item also sold separately.
-• Kiln-dried wood helps prevent warping, splitting and cracking
-• The chairs are solidly constructed using mortise-and-tenon joinery, corner blocks, sturdy solid wood legs, and screwed joints, this piece delivers exceptional stability, longevity, and superior furniture integrity with a 250 lb. weight capacity ensures durability and reliable support for the chair.
-• The chair legs are hand-stained in a natural multi-step black finish to highlight the natural grain and knots of the wood
-• Plastic glides help prevent scratches or mars to floors
-• The chair’s sleek black vegan leather, made from 100% polyester, offers the look and feel of real leather with easy-care convenience.
-• Available in green velvet, brown velvet, beige chenille, gray chenille, white vegan leather and black vegan leather; in counter and dining height sizes
-• Chairs are packed 2 per carton
-• Each marble top is crafted by nature with unique characteristics that vary slightly so no two pieces will be exactly alike
-• 70″ long table seats six comfortably
-• The wood is hand-stained in a natural multi-step black finish to highlight the natural grain and knots of the wood</t>
+          <t>* Expertly crafted of white marble veneers, ash veneers, solid Asian hardwoods and engineered woods, 100% polyester and foam
+* 5-piece set includes the Artemis 70" White Marble Dining Table, Black Finish and 4 Artemis Black Vegan Leather Side Chairs. Each item also sold separately.
+* Kiln-dried wood helps prevent warping, splitting and cracking
+* The chairs are solidly constructed using mortise-and-tenon joinery, corner blocks, sturdy solid wood legs, and screwed joints, this piece delivers exceptional stability, longevity, and superior furniture integrity with a 250 lb. weight capacity ensures durability and reliable support for the chair.
+* The chair legs are hand-stained in a natural multi-step black finish to highlight the natural grain and knots of the wood
+* Plastic glides help prevent scratches or mars to floors
+* The chair's sleek black vegan leather, made from 100% polyester, offers the look and feel of real leather with easy-care convenience.
+* Available in green velvet, brown velvet, beige chenille, gray chenille, white vegan leather and black vegan leather; in counter and dining height sizes
+* Chairs are packed 2 per carton
+* Each marble top is crafted by nature with unique characteristics that vary slightly so no two pieces will be exactly alike
+* 70" long table seats six comfortably
+* The wood is hand-stained in a natural multi-step black finish to highlight the natural grain and knots of the wood</t>
         </is>
       </c>
     </row>
@@ -601,7 +601,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Artemis 5-Piece 70″ Rect White Marble Table, Black Finish w/4 White Vegan Leather Chairs</t>
+          <t>Artemis 5-Piece 70" Rect White Marble Table, Black Finish w/4 White Vegan Leather Chairs</t>
         </is>
       </c>
       <c r="C5" t="inlineStr"/>
@@ -618,23 +618,23 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Meet the Artemis 70-inch marble top table—where modern design feels both elegant and inviting. Its architectural base makes a bold statement, while the sophisticated black finish keeps the look relaxed and livable. The sleek white marble top adds a refined touch. Paired with soft white vegan leather chairs, each with a perfectly pitched seat for comfort, it’s made for gathering. Built with solid wood legs and screwed corner joints, this set offers lasting durability with effortless style.</t>
+          <t>Meet the Artemis 70-inch marble top table-where modern design feels both elegant and inviting. Its architectural base makes a bold statement, while the sophisticated black finish keeps the look relaxed and livable. The sleek white marble top adds a refined touch. Paired with soft white vegan leather chairs, each with a perfectly pitched seat for comfort, it's made for gathering. Built with solid wood legs and screwed corner joints, this set offers lasting durability with effortless style.</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>• Expertly crafted of white marble veneers, ash veneers, solid Asian hardwoods and engineered woods, 100% polyester and foam
-• 5-piece set includes the Artemis 70″ White Marble Dining Table, Black Finish and 4 Artemis White Vegan LeatherSide Chairs. Each item also sold separately.
-• Kiln-dried wood helps prevent warping, splitting and cracking
-• The chairs are solidly constructed using mortise-and-tenon joinery, corner blocks, sturdy solid wood legs, and screwed joints, this piece delivers exceptional stability, longevity, and superior furniture integrity with a 250 lb. weight capacity ensures durability and reliable support for the chair.
-• The chair legs are hand-stained in a natural multi-step black finish to highlight the natural grain and knots of the wood
-• Plastic glides help prevent scratches or mars to floors
-• The chair’s sleek white vegan leather, made from 100% polyester, offers the look and feel of real leather with easy-care convenience.
-• Available in green velvet, brown velvet, beige chenille, gray chenille, white vegan leather and black vegan leather; in counter and dining height sizes
-• Chairs are packed 2 per carton
-• Each marble top is crafted by nature with unique characteristics that vary slightly so no two pieces will be exactly alike
-• 70″ long table seats six comfortably
-• The wood is hand-stained in a natural multi-step black finish to highlight the natural grain and knots of the wood</t>
+          <t>* Expertly crafted of white marble veneers, ash veneers, solid Asian hardwoods and engineered woods, 100% polyester and foam
+* 5-piece set includes the Artemis 70" White Marble Dining Table, Black Finish and 4 Artemis White Vegan LeatherSide Chairs. Each item also sold separately.
+* Kiln-dried wood helps prevent warping, splitting and cracking
+* The chairs are solidly constructed using mortise-and-tenon joinery, corner blocks, sturdy solid wood legs, and screwed joints, this piece delivers exceptional stability, longevity, and superior furniture integrity with a 250 lb. weight capacity ensures durability and reliable support for the chair.
+* The chair legs are hand-stained in a natural multi-step black finish to highlight the natural grain and knots of the wood
+* Plastic glides help prevent scratches or mars to floors
+* The chair's sleek white vegan leather, made from 100% polyester, offers the look and feel of real leather with easy-care convenience.
+* Available in green velvet, brown velvet, beige chenille, gray chenille, white vegan leather and black vegan leather; in counter and dining height sizes
+* Chairs are packed 2 per carton
+* Each marble top is crafted by nature with unique characteristics that vary slightly so no two pieces will be exactly alike
+* 70" long table seats six comfortably
+* The wood is hand-stained in a natural multi-step black finish to highlight the natural grain and knots of the wood</t>
         </is>
       </c>
     </row>
@@ -646,7 +646,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Aubrey 5-Piece 54″ Round Dining Table Set</t>
+          <t>Aubrey 5-Piece 54" Round Dining Table Set</t>
         </is>
       </c>
       <c r="C6" t="inlineStr"/>
@@ -670,21 +670,21 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>• Set includes the Aubrey 54-inch Black Dining Table with Driftwood Stretchers and 4 Aubrey Gray Vegan Leather Side Chairs. Each item also sold separately.
-• Styling details include the dining table with substantial canted 3″ squared posts with contrasting stretchers and exposed tenons that match all the other pieces in the Aubrey collection. Mix and match finishes and pieces within the collection for a custom look.
-• Cross stretchers provide sturdy support and stability for the 54″ Round Table
-• Built with solid wood legs to ensure lasting durability, stability, and timeless elegance for every dining experience.
-• Kiln-dried wood helps prevent warping, splitting, cracking and developing mildew.
-• Plastic glides keep the chair from scratching floor
-• Solidly constructed using mortise-and-tenon joinery and corner blocks for exceptional, longevity, and superior furniture integrity
-• The wood is hand-stained in a natural multi-step black finish with waxed driftwood accents that highlights the natural grain and knots of the wood.
-• Wire-brushed distressing adds depth and character to the chair, making it a truly unique and stylish addition to any space.
-• The chair has a 300 lb. weight capacity to ensure durability and reliable support.
-• Gray vegan leather cover is sleek, durable, and easy-care, adding sophistication to any setting
-• The 54-inch round table seats up to six people
-• Table measurements: 54″W x 54″D x 30″H
-• Chair measurements: 21″W x 22″D x 35.25″H
-• Easy Assembly, all tools included</t>
+          <t>* Set includes the Aubrey 54-inch Black Dining Table with Driftwood Stretchers and 4 Aubrey Gray Vegan Leather Side Chairs. Each item also sold separately.
+* Styling details include the dining table with substantial canted 3" squared posts with contrasting stretchers and exposed tenons that match all the other pieces in the Aubrey collection. Mix and match finishes and pieces within the collection for a custom look.
+* Cross stretchers provide sturdy support and stability for the 54" Round Table
+* Built with solid wood legs to ensure lasting durability, stability, and timeless elegance for every dining experience.
+* Kiln-dried wood helps prevent warping, splitting, cracking and developing mildew.
+* Plastic glides keep the chair from scratching floor
+* Solidly constructed using mortise-and-tenon joinery and corner blocks for exceptional, longevity, and superior furniture integrity
+* The wood is hand-stained in a natural multi-step black finish with waxed driftwood accents that highlights the natural grain and knots of the wood.
+* Wire-brushed distressing adds depth and character to the chair, making it a truly unique and stylish addition to any space.
+* The chair has a 300 lb. weight capacity to ensure durability and reliable support.
+* Gray vegan leather cover is sleek, durable, and easy-care, adding sophistication to any setting
+* The 54-inch round table seats up to six people
+* Table measurements: 54"W x 54"D x 30"H
+* Chair measurements: 21"W x 22"D x 35.25"H
+* Easy Assembly, all tools included</t>
         </is>
       </c>
     </row>
@@ -696,7 +696,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Aubrey 5-Piece 54″ Round Dining Table Set</t>
+          <t>Aubrey 5-Piece 54" Round Dining Table Set</t>
         </is>
       </c>
       <c r="C7" t="inlineStr"/>
@@ -720,22 +720,22 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>• Set includes the Aubrey 54-inch Black Dining Table with Driftwood Stretchers and 4 Aubrey Black Parsons Chairs. Each item also sold separately.
-• Styling details include the dining table with substantial canted 3″ squared posts with contrasting stretchers and exposed tenons that match all the other pieces in the Aubrey collection. Mix and match finishes and pieces within the collection for a custom look.
-• Cross stretchers provide sturdy support and stability for the 54″ Round Table
-• Built with solid wood legs to ensure lasting durability, stability, and timeless elegance for every dining experience.
-• Kiln-dried wood helps prevent warping, splitting, cracking and developing mildew.
-• Plastic glides keep the chair from scratching floor
-• Solidly constructed using mortise-and-tenon joinery and corner blocks for exceptional, longevity, and superior furniture integrity
-• The wood is hand-stained in a natural multi-step black finish with waxed driftwood accents that highlights the natural grain and knots of the wood.
-• Wire-brushed distressing adds depth and character to the chair, making it a truly unique and stylish addition to any space.
-• The chair has a 300 lb. weight capacity to ensure durability and reliable support.
-• The upholstered removable seat is built with 1.1 density foam to offer comfortable seating for the family that is easy to clean, with a versatile design that fits seamlessly into any space, enhancing both comfort and functionality.
-• The chair’s 100% polyester eggshell fabric cover provides a durable and easy-to-clean surface that resists stains and spills.
-• The 54-inch round table seats up to six people
-• Table measurements: 54″W x 54″D x 30″H
-• Chair measurements: 23.5″W x 23.75″D x 38.25″H in
-• Easy Assembly, all tools included</t>
+          <t>* Set includes the Aubrey 54-inch Black Dining Table with Driftwood Stretchers and 4 Aubrey Black Parsons Chairs. Each item also sold separately.
+* Styling details include the dining table with substantial canted 3" squared posts with contrasting stretchers and exposed tenons that match all the other pieces in the Aubrey collection. Mix and match finishes and pieces within the collection for a custom look.
+* Cross stretchers provide sturdy support and stability for the 54" Round Table
+* Built with solid wood legs to ensure lasting durability, stability, and timeless elegance for every dining experience.
+* Kiln-dried wood helps prevent warping, splitting, cracking and developing mildew.
+* Plastic glides keep the chair from scratching floor
+* Solidly constructed using mortise-and-tenon joinery and corner blocks for exceptional, longevity, and superior furniture integrity
+* The wood is hand-stained in a natural multi-step black finish with waxed driftwood accents that highlights the natural grain and knots of the wood.
+* Wire-brushed distressing adds depth and character to the chair, making it a truly unique and stylish addition to any space.
+* The chair has a 300 lb. weight capacity to ensure durability and reliable support.
+* The upholstered removable seat is built with 1.1 density foam to offer comfortable seating for the family that is easy to clean, with a versatile design that fits seamlessly into any space, enhancing both comfort and functionality.
+* The chair's 100% polyester eggshell fabric cover provides a durable and easy-to-clean surface that resists stains and spills.
+* The 54-inch round table seats up to six people
+* Table measurements: 54"W x 54"D x 30"H
+* Chair measurements: 23.5"W x 23.75"D x 38.25"H in
+* Easy Assembly, all tools included</t>
         </is>
       </c>
     </row>
@@ -769,16 +769,16 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>• Constructed of oak and acacia veneers, solid Asian hardwoods and engineered wood
-• Table Top extends from 70 to 88 inches with the insertion of the included 18-inch leaf
-• The Table features a faux plank top with rasping and threading distressing for a relaxed, sophisticated look
-• The Table seats up to eight people when fully extended
-• The chair features a 100% polyester eggshell fabric, offering a durable, easy-to-clean surface that resists stains and spills. A brushed brass accent on the back and distressed greige-finished solid wood legs add a touch of elegance and warmth.
-• The chair also works well as an office or guest chair
-• The optional Sideboard has three deep drawers and one door with metal side drawer glides for smooth operation
-• Set shown included dining table and four Side Chairs. Each piece also sold separately.
-• Oversized brushed brass-tone hardware adds a luxurious touch of elegance and char
-• The wood is hand-stained in a natural multi-step greige finish to highlight the natural grain and knots of the wood</t>
+          <t>* Constructed of oak and acacia veneers, solid Asian hardwoods and engineered wood
+* Table Top extends from 70 to 88 inches with the insertion of the included 18-inch leaf
+* The Table features a faux plank top with rasping and threading distressing for a relaxed, sophisticated look
+* The Table seats up to eight people when fully extended
+* The chair features a 100% polyester eggshell fabric, offering a durable, easy-to-clean surface that resists stains and spills. A brushed brass accent on the back and distressed greige-finished solid wood legs add a touch of elegance and warmth.
+* The chair also works well as an office or guest chair
+* The optional Sideboard has three deep drawers and one door with metal side drawer glides for smooth operation
+* Set shown included dining table and four Side Chairs. Each piece also sold separately.
+* Oversized brushed brass-tone hardware adds a luxurious touch of elegance and char
+* The wood is hand-stained in a natural multi-step greige finish to highlight the natural grain and knots of the wood</t>
         </is>
       </c>
     </row>
@@ -812,15 +812,15 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>• Expertly crafted of acacia veneers, solid Asian hardwoods and engineered wood
-• Table Top extends from 70 to 88 inches with the insertion of the included 18-inch leaf
-• The Table features a faux plank top with rasping and threading distressing for a relaxed, sophisticated look
-• The Table seats up to eight people when fully extended
-• Chair features a relaxed canvas fabric cover application with brushed brass accent on back and distressed toffee finished solid wood legs
-• The chair also works well as an office or guest chair
-• The optional Sideboard has three deep drawers and one door with metal side drawer glides for smooth operation
-• Set shown included dining table and four Side Chairs. Each piece also sold separately.
-• Toffee finish</t>
+          <t>* Expertly crafted of acacia veneers, solid Asian hardwoods and engineered wood
+* Table Top extends from 70 to 88 inches with the insertion of the included 18-inch leaf
+* The Table features a faux plank top with rasping and threading distressing for a relaxed, sophisticated look
+* The Table seats up to eight people when fully extended
+* Chair features a relaxed canvas fabric cover application with brushed brass accent on back and distressed toffee finished solid wood legs
+* The chair also works well as an office or guest chair
+* The optional Sideboard has three deep drawers and one door with metal side drawer glides for smooth operation
+* Set shown included dining table and four Side Chairs. Each piece also sold separately.
+* Toffee finish</t>
         </is>
       </c>
     </row>
@@ -854,15 +854,15 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>• Expertly crafted of acacia veneers, solid Asian hardwoods and engineered wood
-• Kiln-dried wood helps prevent warping, splitting and cracking
-• Two adjustable shelves offer versatile storage options to accommodate items of different sizes and shapes.
-• Includes anti-tip restraint kit for added safety and stability, helping prevent accidental tipping in busy or family spaces.
-• Oversized oil-rubbed brass hardware adds a luxurious touch of elegance and charm
-• Wood scoring and finish rubthrough technique adds a distressed look, enhancing the charm of the furniture with a vintage-inspired appeal.
-• Adjustable levelers add stability on uneven surfaces, protecting contents and enhancing usability
-• Tempered glass doors add durability and safety to the mirror, making it resistant to shattering and damage.
-• The wood is hand-stained in a natural multi-step distressed griege finish to highlight the natural grain and knots of the wood</t>
+          <t>* Expertly crafted of acacia veneers, solid Asian hardwoods and engineered wood
+* Kiln-dried wood helps prevent warping, splitting and cracking
+* Two adjustable shelves offer versatile storage options to accommodate items of different sizes and shapes.
+* Includes anti-tip restraint kit for added safety and stability, helping prevent accidental tipping in busy or family spaces.
+* Oversized oil-rubbed brass hardware adds a luxurious touch of elegance and charm
+* Wood scoring and finish rubthrough technique adds a distressed look, enhancing the charm of the furniture with a vintage-inspired appeal.
+* Adjustable levelers add stability on uneven surfaces, protecting contents and enhancing usability
+* Tempered glass doors add durability and safety to the mirror, making it resistant to shattering and damage.
+* The wood is hand-stained in a natural multi-step distressed griege finish to highlight the natural grain and knots of the wood</t>
         </is>
       </c>
     </row>
@@ -891,16 +891,16 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>The Garland Server marries a modern silohuette with a relaxed, lightly distressed toffee finish in a dining side piece with the perfect casually elegant style of today’s dining rooms. A modern plinth base and tastefully appointed satin brass hardware creates extremely clean lines that displays the natural beauty of the wood expertly. Three drawers and a door allow for plenty of storage base of any dining area in a neat, beautiful package that can stand on its own or can be paired with the matching Garland dining collection.</t>
+          <t>The Garland Server marries a modern silohuette with a relaxed, lightly distressed toffee finish in a dining side piece with the perfect casually elegant style of today's dining rooms. A modern plinth base and tastefully appointed satin brass hardware creates extremely clean lines that displays the natural beauty of the wood expertly. Three drawers and a door allow for plenty of storage base of any dining area in a neat, beautiful package that can stand on its own or can be paired with the matching Garland dining collection.</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>• Constructed of veneers, solids and engineered woods
-• Three deep drawers and one door
-• Metal side drawer guides
-• Medium distressing
-• Toffee finish</t>
+          <t>* Constructed of veneers, solids and engineered woods
+* Three deep drawers and one door
+* Metal side drawer guides
+* Medium distressing
+* Toffee finish</t>
         </is>
       </c>
     </row>
@@ -912,7 +912,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Garland 64″ Sideboard, Greige Finish</t>
+          <t>Garland 64" Sideboard, Greige Finish</t>
         </is>
       </c>
       <c r="C12" t="inlineStr"/>
@@ -934,11 +934,11 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>• Constructed of veneers, solids and engineered woods
-• Three deep drawers and one door
-• Metal side drawer guides
-• Medium distressing
-• Distressed greige finish</t>
+          <t>* Constructed of veneers, solids and engineered woods
+* Three deep drawers and one door
+* Metal side drawer guides
+* Medium distressing
+* Distressed greige finish</t>
         </is>
       </c>
     </row>
@@ -967,24 +967,24 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Modern meets farmhouse in the Magnolia 54-inch Round 5-Piece Dining Set. Large yet intimate, it’s perfect for morning breakfasts or supper club gatherings. The sand and black finish, combined with canted legs forming a sled base, creates a sleek and flowing design. Paired with four solid wood farmhouse chairs, each featuring a shaped solid wood seat, this set remains authentic to its origins while adding a touch of comfort. The Magnolia table comfortably seats six, making it an ideal choice for any dining space.</t>
+          <t>Modern meets farmhouse in the Magnolia 54-inch Round 5-Piece Dining Set. Large yet intimate, it's perfect for morning breakfasts or supper club gatherings. The sand and black finish, combined with canted legs forming a sled base, creates a sleek and flowing design. Paired with four solid wood farmhouse chairs, each featuring a shaped solid wood seat, this set remains authentic to its origins while adding a touch of comfort. The Magnolia table comfortably seats six, making it an ideal choice for any dining space.</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>• Crafted of solid Asian hardwoods, oak veneers and engineered woods
-• The 5-piece set includes the Magnolia black and sand 54-inch round Dining Table and 4 Magnolia Side Chairs. Each item also sold separately.
-• Kiln-dried wood helps prevent warping, splitting, cracking and developing mildew.
-• The chair’s shaped wooden seat adds comfort without compromising classic farmhouse style
-• The chair is corner-blocked and secured with screws for exceptional durability
-• Plastic glides on the chair and table help prevent mars or scratches to floors
-• Built with solid wood legs to ensure lasting durability, stability, and timeless elegance for every dining experience
-• The 54-inch table comfortably seats up to six, enhancing intimate dining experiences with a spacious yet cozy design.
-• The wood is hand-stained in a natural multi-step two-tone sand and black finish to highlight the natural grain and knots of the wood
-• Bottom sled stretchers on the table provide sturdy support and stability for the 54″ Round Table
-• Product Measurements;
- Table: 54″W x 54″D x 30″H
-Side Chair: 20″W x 23″D x 40.25″H</t>
+          <t>* Crafted of solid Asian hardwoods, oak veneers and engineered woods
+* The 5-piece set includes the Magnolia black and sand 54-inch round Dining Table and 4 Magnolia Side Chairs. Each item also sold separately.
+* Kiln-dried wood helps prevent warping, splitting, cracking and developing mildew.
+* The chair's shaped wooden seat adds comfort without compromising classic farmhouse style
+* The chair is corner-blocked and secured with screws for exceptional durability
+* Plastic glides on the chair and table help prevent mars or scratches to floors
+* Built with solid wood legs to ensure lasting durability, stability, and timeless elegance for every dining experience
+* The 54-inch table comfortably seats up to six, enhancing intimate dining experiences with a spacious yet cozy design.
+* The wood is hand-stained in a natural multi-step two-tone sand and black finish to highlight the natural grain and knots of the wood
+* Bottom sled stretchers on the table provide sturdy support and stability for the 54" Round Table
+* Product Measurements;
+ Table: 54"W x 54"D x 30"H
+Side Chair: 20"W x 23"D x 40.25"H</t>
         </is>
       </c>
     </row>
@@ -1018,16 +1018,16 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>• Crafted from oak veneers, Asian hardwood solids and engineered woods
-• Cathedral glass door fronts offer a beautiful display area or excellent remote access for electronics
-• Contrasting weathered sand interior beautifully accents the interior with the contrasting ebony finished exterior
-• Two adjustable shelves offer versatile storage options to accommodate items of different sizes and shapes.
-• Wire escape back with notched shelves ensures organized cable management and a clutter-free appearance
-• With wire management and cathedral glass doors, the Server can work as a dining room Server, a living room entertainment piece or a hallway or foyer console.
-• The wood is hand-stained in a natural multi-step weathered sand finish with black interior to highlight the interior of the case while offering a beautiful contrast
-• 200 lb. weight capacity ensures durability and reliable support.
-• Adjustable levelers add stability on uneven floors
-• The black accented interior and weathered sand exterior allows seamless style integration with all elements of the Magnolia collection</t>
+          <t>* Crafted from oak veneers, Asian hardwood solids and engineered woods
+* Cathedral glass door fronts offer a beautiful display area or excellent remote access for electronics
+* Contrasting weathered sand interior beautifully accents the interior with the contrasting ebony finished exterior
+* Two adjustable shelves offer versatile storage options to accommodate items of different sizes and shapes.
+* Wire escape back with notched shelves ensures organized cable management and a clutter-free appearance
+* With wire management and cathedral glass doors, the Server can work as a dining room Server, a living room entertainment piece or a hallway or foyer console.
+* The wood is hand-stained in a natural multi-step weathered sand finish with black interior to highlight the interior of the case while offering a beautiful contrast
+* 200 lb. weight capacity ensures durability and reliable support.
+* Adjustable levelers add stability on uneven floors
+* The black accented interior and weathered sand exterior allows seamless style integration with all elements of the Magnolia collection</t>
         </is>
       </c>
     </row>
@@ -1056,20 +1056,20 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>A masterpiece of style and versatility, the Magnolia Server transforms any room with its bold dusty blue finish and weathered sand interior. Elegant Cathedral glass doors reveal adjustable shelves for display, while hidden cable management ensures seamless integration. Whether as a sideboard, entertainment center, or hallway console, it blends practicality with sophistication. Clean lines and thoughtful details enhance both style and storage, making it a refined choice for any home—offering modern elegance with functionality in every setting.</t>
+          <t>A masterpiece of style and versatility, the Magnolia Server transforms any room with its bold dusty blue finish and weathered sand interior. Elegant Cathedral glass doors reveal adjustable shelves for display, while hidden cable management ensures seamless integration. Whether as a sideboard, entertainment center, or hallway console, it blends practicality with sophistication. Clean lines and thoughtful details enhance both style and storage, making it a refined choice for any home-offering modern elegance with functionality in every setting.</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>• Crafted from oak veneers, Asian hardwood solids and engineered woods
-• Cathedral glass door fronts offer a beautiful display area or excellent remote access for electronics
-• Contrasting weathered sand interior beautifully accents the interior with the contrasting dusty blue finished exterior
-• Two adjustable shelves offer versatile storage options to accommodate items of different sizes and shapes.
-• Wire escape back with notched shelves ensures organized cable management and a clutter-free appearance
-• With wire management and cathedral glass doors, the Server can work as a dining room Server, a living room entertainment piece or a hallway or foyer console.
-• The wood is hand-stained in a natural multi-step dusty blue finish with weathered sand interior to highlight the interior of the case while offering a beautiful contrast
-• 200 lb. weight capacity ensures durability and reliable support.
-• Adjustable levelers add stability on uneven floors</t>
+          <t>* Crafted from oak veneers, Asian hardwood solids and engineered woods
+* Cathedral glass door fronts offer a beautiful display area or excellent remote access for electronics
+* Contrasting weathered sand interior beautifully accents the interior with the contrasting dusty blue finished exterior
+* Two adjustable shelves offer versatile storage options to accommodate items of different sizes and shapes.
+* Wire escape back with notched shelves ensures organized cable management and a clutter-free appearance
+* With wire management and cathedral glass doors, the Server can work as a dining room Server, a living room entertainment piece or a hallway or foyer console.
+* The wood is hand-stained in a natural multi-step dusty blue finish with weathered sand interior to highlight the interior of the case while offering a beautiful contrast
+* 200 lb. weight capacity ensures durability and reliable support.
+* Adjustable levelers add stability on uneven floors</t>
         </is>
       </c>
     </row>
@@ -1103,13 +1103,13 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>• Constructed of mango and Asian hardwoods, mango veneers and engineered hardwoods
-• Side Chair features schoolhouse design with shaped top rail and upholstered linen-colored seat for comfort
-• The table has plank-effect top, double pedestal base with exposed tenons
-• Stretchers on the table base add to the stability and strength of the table
-• Table seats up to 10 with two 18-inch leaves inserted
-• Table extension slides use cables to guarantee a smooth, seamless leaf insert operation, reducing wear and safeguarding against potential jamming or misalignment
-• Dusky cedar finish</t>
+          <t>* Constructed of mango and Asian hardwoods, mango veneers and engineered hardwoods
+* Side Chair features schoolhouse design with shaped top rail and upholstered linen-colored seat for comfort
+* The table has plank-effect top, double pedestal base with exposed tenons
+* Stretchers on the table base add to the stability and strength of the table
+* Table seats up to 10 with two 18-inch leaves inserted
+* Table extension slides use cables to guarantee a smooth, seamless leaf insert operation, reducing wear and safeguarding against potential jamming or misalignment
+* Dusky cedar finish</t>
         </is>
       </c>
     </row>
@@ -1138,25 +1138,25 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>The Reid 5-Piece Dining Set blends modern style with everyday versatility, featuring the Reid 77–95″ Dining Table and four coordinating side chairs. The table expands with an 18-inch leaf to seat up to eight and showcases a deep black finish for a neutral accent to any room. Reid chairs add tailored comfort with box-pleat seats, foam cushioning, and easy-care saddle brown vegan leather. An exposed webbed back and angled seat provide relaxed support, making this set ideal for dining, entertaining, or casual gatherings.</t>
+          <t>The Reid 5-Piece Dining Set blends modern style with everyday versatility, featuring the Reid 77-95" Dining Table and four coordinating side chairs. The table expands with an 18-inch leaf to seat up to eight and showcases a deep black finish for a neutral accent to any room. Reid chairs add tailored comfort with box-pleat seats, foam cushioning, and easy-care saddle brown vegan leather. An exposed webbed back and angled seat provide relaxed support, making this set ideal for dining, entertaining, or casual gatherings.</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>• Expertly crafted of ash veneers, solid Asian hardwoods, vegan leather, foam and engineered woods
-• 5-Piece Set includes the Reid 77-95″ Dining Table with 18-inch leaf and 4 Reid Saddle Brown Vegan Leather Side Chairs. Each item also sold separately.
-• Table expands from 77″ to 95″ with included leaf to seat up to eight
-• Hand-stained multi-step sand finish highlights natural grain and knots
-• Experience affordable, leather-like luxury with the camel vegan leather chair from 20% polyurethane/80% polyester that’s easy to care for, comfortable, and adds a warm, rustic leather-like touch to your dining space.
-• Solid construction with mortise-and-tenon joinery, corner blocks, stretchers, and reinforced joints
-• Plastic glides help protect floors from scratches
-• 300 lb. weight capacity per chair for reliable support
-• Easy assembly with all tools included
-• Product Measurements:
+          <t>* Expertly crafted of ash veneers, solid Asian hardwoods, vegan leather, foam and engineered woods
+* 5-Piece Set includes the Reid 77-95" Dining Table with 18-inch leaf and 4 Reid Saddle Brown Vegan Leather Side Chairs. Each item also sold separately.
+* Table expands from 77" to 95" with included leaf to seat up to eight
+* Hand-stained multi-step sand finish highlights natural grain and knots
+* Experience affordable, leather-like luxury with the camel vegan leather chair from 20% polyurethane/80% polyester that's easy to care for, comfortable, and adds a warm, rustic leather-like touch to your dining space.
+* Solid construction with mortise-and-tenon joinery, corner blocks, stretchers, and reinforced joints
+* Plastic glides help protect floors from scratches
+* 300 lb. weight capacity per chair for reliable support
+* Easy assembly with all tools included
+* Product Measurements:
  Table: 77-95W x 40D x 30
-• Side Chair: 20W x 24.25D x 40H
-• Chair Fabric Content: 20% polyurethane, 80% polyester
-• Cleaning Code: W — Easy-care vegan leather wipes clean with mild soap and water, offering durable style that stands up to everyday use and spills.</t>
+* Side Chair: 20W x 24.25D x 40H
+* Chair Fabric Content: 20% polyurethane, 80% polyester
+* Cleaning Code: W - Easy-care vegan leather wipes clean with mild soap and water, offering durable style that stands up to everyday use and spills.</t>
         </is>
       </c>
     </row>
@@ -1168,7 +1168,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Reid 5-Piece 77-95″ Dining Set, Sand Finish with Camel Vegan Leather</t>
+          <t>Reid 5-Piece 77-95" Dining Set, Sand Finish with Camel Vegan Leather</t>
         </is>
       </c>
       <c r="C18" t="inlineStr"/>
@@ -1185,25 +1185,25 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>The Reid 5-Piece Dining Set blends modern style with everyday versatility, featuring the Reid 77–95″ Dining Table and four coordinating side chairs. The table expands with an 18-inch leaf to seat up to eight and showcases a light sand finish that highlights natural wood grain. Reid chairs add tailored comfort with box-pleat seats, foam cushioning, and easy-care camel vegan leather. An exposed webbed back and angled seat provide relaxed support, making this set ideal for dining, entertaining, or casual gatherings.</t>
+          <t>The Reid 5-Piece Dining Set blends modern style with everyday versatility, featuring the Reid 77-95" Dining Table and four coordinating side chairs. The table expands with an 18-inch leaf to seat up to eight and showcases a light sand finish that highlights natural wood grain. Reid chairs add tailored comfort with box-pleat seats, foam cushioning, and easy-care camel vegan leather. An exposed webbed back and angled seat provide relaxed support, making this set ideal for dining, entertaining, or casual gatherings.</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>• Expertly crafted of ash veneers, solid Asian hardwoods, vegan leather, foam and engineered woods
-• 5-Piece Set includes the Reid 77-95″ Dining Table with 18-inch leaf and 4 Reid Camel Vegan Leather Side Chairs. Each item also sold separately.
-• Table expands from 77″ to 95″ with included leaf to seat up to eight
-• Hand-stained multi-step sand finish highlights natural grain and knots
-• Experience affordable, leather-like luxury with the camel vegan leather chair from 60% polyurethane/40% polyester that’s easy to care for, comfortable, and adds a warm, rustic leather-like touch to your dining space.
-• Solid construction with mortise-and-tenon joinery, corner blocks, stretchers, and reinforced joints
-• Plastic glides help protect floors from scratches
-• 300 lb. weight capacity per chair for reliable support
-• Easy assembly with all tools included
-• Product Measurements:
+          <t>* Expertly crafted of ash veneers, solid Asian hardwoods, vegan leather, foam and engineered woods
+* 5-Piece Set includes the Reid 77-95" Dining Table with 18-inch leaf and 4 Reid Camel Vegan Leather Side Chairs. Each item also sold separately.
+* Table expands from 77" to 95" with included leaf to seat up to eight
+* Hand-stained multi-step sand finish highlights natural grain and knots
+* Experience affordable, leather-like luxury with the camel vegan leather chair from 60% polyurethane/40% polyester that's easy to care for, comfortable, and adds a warm, rustic leather-like touch to your dining space.
+* Solid construction with mortise-and-tenon joinery, corner blocks, stretchers, and reinforced joints
+* Plastic glides help protect floors from scratches
+* 300 lb. weight capacity per chair for reliable support
+* Easy assembly with all tools included
+* Product Measurements:
  Table: 77-95W x 40D x 30
-• Side Chair: 20W x 24.25D x 40H
-• Chair Fabric Content: 60% polyurethane, 40% polyester
-• Cleaning Code: W — Easy-care vegan leather wipes clean with mild soap and water, offering durable style that stands up to everyday use and spills.</t>
+* Side Chair: 20W x 24.25D x 40H
+* Chair Fabric Content: 60% polyurethane, 40% polyester
+* Cleaning Code: W - Easy-care vegan leather wipes clean with mild soap and water, offering durable style that stands up to everyday use and spills.</t>
         </is>
       </c>
     </row>
@@ -1215,7 +1215,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Reid 60″ Server, Black Finish</t>
+          <t>Reid 60" Server, Black Finish</t>
         </is>
       </c>
       <c r="C19" t="inlineStr"/>
@@ -1232,22 +1232,22 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>The Reid 60″ Server offers a modern take on a versatile dining and entertainment piece. Its rich midnight black finish over ash veneers delivers a bold, refined look for any room. Two glass doors provide display, storage, and easy remote access, while two adjustable interior shelves customize space for décor or electronics. Convenient charging is built in with two electric outlets plus USB-A and USB-C ports on the outer upper back, paired with a wire escape for organized cords. Clean lines complete the look overall.</t>
+          <t>The Reid 60" Server offers a modern take on a versatile dining and entertainment piece. Its rich midnight black finish over ash veneers delivers a bold, refined look for any room. Two glass doors provide display, storage, and easy remote access, while two adjustable interior shelves customize space for décor or electronics. Convenient charging is built in with two electric outlets plus USB-A and USB-C ports on the outer upper back, paired with a wire escape for organized cords. Clean lines complete the look overall.</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>• Expertly crafted of ash veneers, solid Asian hardwoods and engineered woods
-• Kiln-dried wood helps prevent warping, splitting and cracking
-• Two adjustable shelves offer versatile storage options to accommodate items of different sizes and shapes.
-• A built-in wire escape with integrated electric and USB-A/C outlets on the upper outside back keeps cords organized and devices conveniently powered while maintaining a clean look.
-• Concealed European hinges offer clean front aesthetic while allowing the doors to open and close smoothly and quietly
-• Finished back allows for seamless placement in any space.
-• The wood is hand-stained in a natural multi-step black finish to highlight the natural grain and knots of the wood
-• Easy Assembly, all tools included
-• 200 lb. weight capacity ensures durability and reliable support.
-• Oversized brass colored hardware adds a luxurious touch of elegance and charm
-• Includes anti-tip restraint kit for added safety and stability, helping prevent accidental tipping in busy or family spaces.</t>
+          <t>* Expertly crafted of ash veneers, solid Asian hardwoods and engineered woods
+* Kiln-dried wood helps prevent warping, splitting and cracking
+* Two adjustable shelves offer versatile storage options to accommodate items of different sizes and shapes.
+* A built-in wire escape with integrated electric and USB-A/C outlets on the upper outside back keeps cords organized and devices conveniently powered while maintaining a clean look.
+* Concealed European hinges offer clean front aesthetic while allowing the doors to open and close smoothly and quietly
+* Finished back allows for seamless placement in any space.
+* The wood is hand-stained in a natural multi-step black finish to highlight the natural grain and knots of the wood
+* Easy Assembly, all tools included
+* 200 lb. weight capacity ensures durability and reliable support.
+* Oversized brass colored hardware adds a luxurious touch of elegance and charm
+* Includes anti-tip restraint kit for added safety and stability, helping prevent accidental tipping in busy or family spaces.</t>
         </is>
       </c>
     </row>
@@ -1259,7 +1259,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Reid 60″ Server, Sand Finish</t>
+          <t>Reid 60" Server, Sand Finish</t>
         </is>
       </c>
       <c r="C20" t="inlineStr"/>
@@ -1276,23 +1276,23 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>The Reid 60″ Server offers a modern take on a versatile dining and entertainment piece. Its light, airy sand finish over ash veneers brings a fresh, open feel to any room. Two glass doors provide display, storage, and easy remote access, while two adjustable interior shelves customize space for décor or electronics. Convenient charging is built in with two electric outlets plus USB-A and USB-C ports on the outer upper back, paired with a wire escape for organized cords. Clean lines complete the look overall.</t>
+          <t>The Reid 60" Server offers a modern take on a versatile dining and entertainment piece. Its light, airy sand finish over ash veneers brings a fresh, open feel to any room. Two glass doors provide display, storage, and easy remote access, while two adjustable interior shelves customize space for décor or electronics. Convenient charging is built in with two electric outlets plus USB-A and USB-C ports on the outer upper back, paired with a wire escape for organized cords. Clean lines complete the look overall.</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>• Expertly crafted of ash veneers, solid Asian hardwoods and engineered woods
-• Kiln-dried wood helps prevent warping, splitting and cracking
-• Two adjustable shelves offer versatile storage options to accommodate items of different sizes and shapes.
-• A built-in wire escape with integrated electric and USB-A/C outlets on the upper outside back keeps cords organized and devices conveniently powered while maintaining a clean look.
-• Adjustable levelers add stability on uneven floors
-• Concealed European hinges offer clean front aesthetic while allowing the doors to open and close smoothly and quietly
-• Finished back allows for seamless placement in any space.
-• The wood is hand-stained in a natural multi-step sand finish to highlight the natural grain and knots of the wood
-• Easy Assembly, all tools included
-• 200 lb. weight capacity ensures durability and reliable support.
-• Oversized brass colored hardware adds a luxurious touch of elegance and charm
-• Includes anti-tip restraint kit for added safety and stability, helping prevent accidental tipping in busy or family spaces.</t>
+          <t>* Expertly crafted of ash veneers, solid Asian hardwoods and engineered woods
+* Kiln-dried wood helps prevent warping, splitting and cracking
+* Two adjustable shelves offer versatile storage options to accommodate items of different sizes and shapes.
+* A built-in wire escape with integrated electric and USB-A/C outlets on the upper outside back keeps cords organized and devices conveniently powered while maintaining a clean look.
+* Adjustable levelers add stability on uneven floors
+* Concealed European hinges offer clean front aesthetic while allowing the doors to open and close smoothly and quietly
+* Finished back allows for seamless placement in any space.
+* The wood is hand-stained in a natural multi-step sand finish to highlight the natural grain and knots of the wood
+* Easy Assembly, all tools included
+* 200 lb. weight capacity ensures durability and reliable support.
+* Oversized brass colored hardware adds a luxurious touch of elegance and charm
+* Includes anti-tip restraint kit for added safety and stability, helping prevent accidental tipping in busy or family spaces.</t>
         </is>
       </c>
     </row>
@@ -1321,30 +1321,30 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Dive into a mix of classic fun and modern chic with the Rylie Folding Game Counter Dining Set. This natural finished set features swivel Captain’s Chairs in camel vegan leather, accented with stylish copper nailheads. The star is the removable game top, decked out with 16 cupholders and eight chip holders for ultimate game nights. Post-play, it transforms into a charming dining spot. Crafted from durable oak veneers and hardwoods, this set seats four comfortably and assembles easily, making it a perfect blend of form and function.</t>
+          <t>Dive into a mix of classic fun and modern chic with the Rylie Folding Game Counter Dining Set. This natural finished set features swivel Captain's Chairs in camel vegan leather, accented with stylish copper nailheads. The star is the removable game top, decked out with 16 cupholders and eight chip holders for ultimate game nights. Post-play, it transforms into a charming dining spot. Crafted from durable oak veneers and hardwoods, this set seats four comfortably and assembles easily, making it a perfect blend of form and function.</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>• Set includes the Rylie Folding Game Top, the Rylie 48-inch Counter Dining Table and 4 Rylie Counter Captains Chairs. All in natural finish with camel vegan leather. Each item also sold separately..
-• Expertly crafted of oak veneers, poplar and Asian hardwood solids and engineered woods, foam and vegan leather
-• Kiln-dried wood helps prevent warping, splitting, cracking and developing mildew.
-• The removable Folding Game Top has 16 cupholders and eight chip holders make for great multi-player game entertainment
-• Folding game top sits on top of the 48-inch round Rylie table for game night and then can be removed and stored in the included carry bag to use the table for dining
-• Four undertop felt-lined drawers offer additional storage for dining or game essentials
-• The 48-inch round table fosters a cozy, intimate setting, perfect for close-knit gatherings and conversations.
-• The 36-inch Counter Height Table offers versatility for dining or working, perfectly suited for standing activities.
-• Beautiful inlaid pinwheel oak veneer pattern creates a stunning work or dining surface
-• Table seats up to four comfortably
-• Adjustable levelers add stability on uneven surfaces.
-• 360-degree swivel mechanism provides greater mobility, reduces strain on the body, and adds an element of playfulness to your decor.
-• Built with solid wood legs to ensure lasting durability, stability, and timeless elegance for every dining experience.
-• The camel colored vegan leather counter chair, accented with copper nailhead trim, offers a sophisticated look with the soft touch and durability of leather, yet is easy to maintain and resistant to wear and tear
-• The Counter Stool’s 24-inch high seat effortlessly complements 36-inch high counters, ensuring an ideal seating experience.
-• Front and side stretchers provide sturdy support and stability for the 24″ seat height counter stool
-• The wood is hand-stained in a multi-step natural glaze that beautifully highlights the natural grain and knots of the wood
-• Fabric Content: in 69% polyurethane, 28% polyester and 3% viscose
-• Easy Assembly, all tools included</t>
+          <t>* Set includes the Rylie Folding Game Top, the Rylie 48-inch Counter Dining Table and 4 Rylie Counter Captains Chairs. All in natural finish with camel vegan leather. Each item also sold separately..
+* Expertly crafted of oak veneers, poplar and Asian hardwood solids and engineered woods, foam and vegan leather
+* Kiln-dried wood helps prevent warping, splitting, cracking and developing mildew.
+* The removable Folding Game Top has 16 cupholders and eight chip holders make for great multi-player game entertainment
+* Folding game top sits on top of the 48-inch round Rylie table for game night and then can be removed and stored in the included carry bag to use the table for dining
+* Four undertop felt-lined drawers offer additional storage for dining or game essentials
+* The 48-inch round table fosters a cozy, intimate setting, perfect for close-knit gatherings and conversations.
+* The 36-inch Counter Height Table offers versatility for dining or working, perfectly suited for standing activities.
+* Beautiful inlaid pinwheel oak veneer pattern creates a stunning work or dining surface
+* Table seats up to four comfortably
+* Adjustable levelers add stability on uneven surfaces.
+* 360-degree swivel mechanism provides greater mobility, reduces strain on the body, and adds an element of playfulness to your decor.
+* Built with solid wood legs to ensure lasting durability, stability, and timeless elegance for every dining experience.
+* The camel colored vegan leather counter chair, accented with copper nailhead trim, offers a sophisticated look with the soft touch and durability of leather, yet is easy to maintain and resistant to wear and tear
+* The Counter Stool's 24-inch high seat effortlessly complements 36-inch high counters, ensuring an ideal seating experience.
+* Front and side stretchers provide sturdy support and stability for the 24" seat height counter stool
+* The wood is hand-stained in a multi-step natural glaze that beautifully highlights the natural grain and knots of the wood
+* Fabric Content: in 69% polyurethane, 28% polyester and 3% viscose
+* Easy Assembly, all tools included</t>
         </is>
       </c>
     </row>
@@ -1373,28 +1373,28 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Get ready for game night with the Rylie Black Finish 6-Piece Game Dining Set! This set includes a 48-inch round table with a folding game top and four comfy castered Captain’s chairs in sand vegan leather, jazzed up with copper nailhead trim. The folding game top offers eight stations with dual cupholders and chip holders. When the games are done, remove the top, tuck it away in its carry case, and you’ve got a sleek dining table ready for four.
+          <t>Get ready for game night with the Rylie Black Finish 6-Piece Game Dining Set! This set includes a 48-inch round table with a folding game top and four comfy castered Captain's chairs in sand vegan leather, jazzed up with copper nailhead trim. The folding game top offers eight stations with dual cupholders and chip holders. When the games are done, remove the top, tuck it away in its carry case, and you've got a sleek dining table ready for four.
  The glossy black finish gives it a modern edge, perfect for any room. Each piece is crafted from oak veneers, poplar, and Asian hardwoods, kiln-dried to avoid warping or mildew. The pinwheel oak veneer pattern on the table adds elegance, making it great for dining or working. The chairs, with full rotation and solid wood legs, are stylish and practical.</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>• Set includes the Rylie 48-inch round table top, the Rylie Trestle Table Base, Folding Game Table Top and 4 Black Captains Chair. Each item also sold separately.
-• Crafted of oak veneers, poplar and Asian hardwood solids and engineered woods
-• Kiln-dried wood helps prevent warping, splitting, cracking and developing mildew.
-• Removable Folding Game Top has 16 cupholders and eight chip holders make for great multi-player game entertainment
-• Folding Game Top sits on top of the 48-inch round Rylie table for game night and then can be removed and stored in the included carry bag to use the table for dining
-• The 48-inch round table fosters a cozy, intimate setting, perfect for close-knit gatherings and conversations.
-• Beautiful inlaid pinwheel oak veneer pattern creates a stunning work or dining surface
-• Table seats up to four comfortably
-• Versatile side chair suitable for dining, office, or living areas, serving as a stylish accent piece
-• Fully rotating casters on the chair offer enhanced mobility and convenience, allowing for smooth, effortless movement across various floor surfaces
-• Chair is built with solid wood legs to ensure lasting durability, stability, and timeless elegance for every dining experience.
-• The sand colored vegan leather chair, accented with copper nailhead trim, offers a sophisticated look with the soft touch and durability of leather, yet is easy to maintain and resistant to wear and tear
-• The wood is hand-stained in a natural multi-step glossy black finish to highlight the natural grain and knots of the wood
-• Fabric Content: in 69% polyurethane, 28% polyester and 3% viscose
-• Adjustable levelers add stability on uneven surfaces.
-• Easy Assembly, all tools included</t>
+          <t>* Set includes the Rylie 48-inch round table top, the Rylie Trestle Table Base, Folding Game Table Top and 4 Black Captains Chair. Each item also sold separately.
+* Crafted of oak veneers, poplar and Asian hardwood solids and engineered woods
+* Kiln-dried wood helps prevent warping, splitting, cracking and developing mildew.
+* Removable Folding Game Top has 16 cupholders and eight chip holders make for great multi-player game entertainment
+* Folding Game Top sits on top of the 48-inch round Rylie table for game night and then can be removed and stored in the included carry bag to use the table for dining
+* The 48-inch round table fosters a cozy, intimate setting, perfect for close-knit gatherings and conversations.
+* Beautiful inlaid pinwheel oak veneer pattern creates a stunning work or dining surface
+* Table seats up to four comfortably
+* Versatile side chair suitable for dining, office, or living areas, serving as a stylish accent piece
+* Fully rotating casters on the chair offer enhanced mobility and convenience, allowing for smooth, effortless movement across various floor surfaces
+* Chair is built with solid wood legs to ensure lasting durability, stability, and timeless elegance for every dining experience.
+* The sand colored vegan leather chair, accented with copper nailhead trim, offers a sophisticated look with the soft touch and durability of leather, yet is easy to maintain and resistant to wear and tear
+* The wood is hand-stained in a natural multi-step glossy black finish to highlight the natural grain and knots of the wood
+* Fabric Content: in 69% polyurethane, 28% polyester and 3% viscose
+* Adjustable levelers add stability on uneven surfaces.
+* Easy Assembly, all tools included</t>
         </is>
       </c>
     </row>
@@ -1423,29 +1423,29 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>The Rylie 6-piece Game Dining Set presents a versatile ensemble for both game nights and stylish dining. This set includes the Rylie Folding Game Table Top, a 48-inch round Dining Table, and four Rylie castered Captain’s Chairs in a natural finish with camel vegan leather. Each piece, available separately, is crafted from oak veneers, poplar, and Asian hardwoods, ensuring durability and resistance to warping or mildew.
- The game top, featuring 16 cupholders and eight chip holders, easily transforms your dining table into a multi-player game station. Post-game, simply store the top in its carry bag to reveal a stunning dining surface with an inlaid pinwheel oak veneer pattern. The table’s natural finish highlights the wood’s grain, creating a warm, inviting setting for up to four people. The chairs, with full rotation casters, offer seamless mobility and comfort, accented with copper nailhead trim for an elegant touch. This set combines practicality with elegance, ideal for any home. Easy assembly with all tools included.</t>
+          <t>The Rylie 6-piece Game Dining Set presents a versatile ensemble for both game nights and stylish dining. This set includes the Rylie Folding Game Table Top, a 48-inch round Dining Table, and four Rylie castered Captain's Chairs in a natural finish with camel vegan leather. Each piece, available separately, is crafted from oak veneers, poplar, and Asian hardwoods, ensuring durability and resistance to warping or mildew.
+ The game top, featuring 16 cupholders and eight chip holders, easily transforms your dining table into a multi-player game station. Post-game, simply store the top in its carry bag to reveal a stunning dining surface with an inlaid pinwheel oak veneer pattern. The table's natural finish highlights the wood's grain, creating a warm, inviting setting for up to four people. The chairs, with full rotation casters, offer seamless mobility and comfort, accented with copper nailhead trim for an elegant touch. This set combines practicality with elegance, ideal for any home. Easy assembly with all tools included.</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>• Set includes the Rylie Folding Game Table Top, the Rylie 48-inch round Dining Table and 4 Rylie castered Captains Chairs in natural finish with camel vegan leather. Each item also sold separately.
-• Crafted of oak veneers, poplar and Asian hardwood solids and engineered woods
-• Kiln-dried wood helps prevent warping, splitting, cracking and developing mildew.
-• Removable Folding Game Top has 16 cupholders and eight chip holders make for great multi-player game entertainment
-• Folding Game Top sits on top of the 48-inch round Rylie table for game night and then can be removed and stored in the included carry bag to use the table for dining
-• The 48-inch round table fosters a cozy, intimate setting, perfect for close-knit gatherings and conversations.
-• The wood is hand-stained in a natural multi-step natural finish that beautifully highlights the natural grain and knots of the wood
-• Beautiful inlaid pinwheel oak veneer pattern creates a stunning work or dining surface
-• Table seats up to four comfortably
-• Versatile side chair suitable for dining, office, or living areas, serving as a stylish accent piece
-• Fully rotating casters on the chair offer enhanced mobility and convenience, allowing for smooth, effortless movement across various floor surfaces
-• Chair is built with solid wood legs to ensure lasting durability, stability, and timeless elegance for every dining experience.
-• The sand colored vegan leather chair, accented with copper nailhead trim, offers a sophisticated look with the soft touch and durability of leather, yet is easy to maintain and resistant to wear and tear
-• The wood is hand-stained in a natural multi-step glossy black finish to highlight the natural grain and knots of the wood
-• Fabric Content: in 69% polyurethane, 28% polyester and 3% viscose
-• Adjustable levelers add stability on uneven surfaces.
-• Easy Assembly, all tools included</t>
+          <t>* Set includes the Rylie Folding Game Table Top, the Rylie 48-inch round Dining Table and 4 Rylie castered Captains Chairs in natural finish with camel vegan leather. Each item also sold separately.
+* Crafted of oak veneers, poplar and Asian hardwood solids and engineered woods
+* Kiln-dried wood helps prevent warping, splitting, cracking and developing mildew.
+* Removable Folding Game Top has 16 cupholders and eight chip holders make for great multi-player game entertainment
+* Folding Game Top sits on top of the 48-inch round Rylie table for game night and then can be removed and stored in the included carry bag to use the table for dining
+* The 48-inch round table fosters a cozy, intimate setting, perfect for close-knit gatherings and conversations.
+* The wood is hand-stained in a natural multi-step natural finish that beautifully highlights the natural grain and knots of the wood
+* Beautiful inlaid pinwheel oak veneer pattern creates a stunning work or dining surface
+* Table seats up to four comfortably
+* Versatile side chair suitable for dining, office, or living areas, serving as a stylish accent piece
+* Fully rotating casters on the chair offer enhanced mobility and convenience, allowing for smooth, effortless movement across various floor surfaces
+* Chair is built with solid wood legs to ensure lasting durability, stability, and timeless elegance for every dining experience.
+* The sand colored vegan leather chair, accented with copper nailhead trim, offers a sophisticated look with the soft touch and durability of leather, yet is easy to maintain and resistant to wear and tear
+* The wood is hand-stained in a natural multi-step glossy black finish to highlight the natural grain and knots of the wood
+* Fabric Content: in 69% polyurethane, 28% polyester and 3% viscose
+* Adjustable levelers add stability on uneven surfaces.
+* Easy Assembly, all tools included</t>
         </is>
       </c>
     </row>
@@ -1480,14 +1480,14 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>• Crafted from Oak veneers, Asian hardwood solids and engineered woods
-• Wire Escape back allows this cabinet to double as a media console
-• Cathedral glass door fronts offer a beautiful display area or excellent remote access  for electronics
-• Contrasting black interior beautifully accents the interior with the contrasting cocoa finished exterior
-• Two adjustable shelves offer versatile storage options to accommodate items of different sizes and shapes.
-• Wire escape back with notched shelves ensures organized cable management and a clutter-free appearance
-• With wire management and cathedral glass doors, the Server can work as a dining room Server, a living room entertainment piece or a hallway or foyer console.
-• The wood is hand-stained in a natural multi-step cocoa finish with black  interior to highlight the interior of the case while offering a beautiful contrast</t>
+          <t>* Crafted from Oak veneers, Asian hardwood solids and engineered woods
+* Wire Escape back allows this cabinet to double as a media console
+* Cathedral glass door fronts offer a beautiful display area or excellent remote access  for electronics
+* Contrasting black interior beautifully accents the interior with the contrasting cocoa finished exterior
+* Two adjustable shelves offer versatile storage options to accommodate items of different sizes and shapes.
+* Wire escape back with notched shelves ensures organized cable management and a clutter-free appearance
+* With wire management and cathedral glass doors, the Server can work as a dining room Server, a living room entertainment piece or a hallway or foyer console.
+* The wood is hand-stained in a natural multi-step cocoa finish with black  interior to highlight the interior of the case while offering a beautiful contrast</t>
         </is>
       </c>
     </row>

</xml_diff>